<commit_message>
Se realizan ajustes en portas, preactivador y legalizador para que implementen el autologin y los tiempos random entre cada transaccion
</commit_message>
<xml_diff>
--- a/src/portas/portabilidad.xlsx
+++ b/src/portas/portabilidad.xlsx
@@ -3994,10 +3994,14 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L66" t="inlineStr"/>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>54386419</t>
+        </is>
+      </c>
       <c r="M66" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>129.91</t>
         </is>
       </c>
       <c r="N66" t="inlineStr"/>
@@ -4044,8 +4048,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L67" t="inlineStr"/>
-      <c r="M67" t="inlineStr"/>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>54386457</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>119.8</t>
+        </is>
+      </c>
       <c r="N67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -4198,8 +4210,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L70" t="inlineStr"/>
-      <c r="M70" t="inlineStr"/>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>54386499</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>118.9</t>
+        </is>
+      </c>
       <c r="N70" t="inlineStr"/>
     </row>
     <row r="71">
@@ -4298,8 +4318,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L72" t="inlineStr"/>
-      <c r="M72" t="inlineStr"/>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>54386552</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>129.41</t>
+        </is>
+      </c>
       <c r="N72" t="inlineStr"/>
     </row>
     <row r="73">
@@ -4344,8 +4372,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L73" t="inlineStr"/>
-      <c r="M73" t="inlineStr"/>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>54386594</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>131.46</t>
+        </is>
+      </c>
       <c r="N73" t="inlineStr"/>
     </row>
     <row r="74">
@@ -4390,8 +4426,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L74" t="inlineStr"/>
-      <c r="M74" t="inlineStr"/>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>54386654</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>120.43</t>
+        </is>
+      </c>
       <c r="N74" t="inlineStr"/>
     </row>
     <row r="75">
@@ -4436,8 +4480,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L75" t="inlineStr"/>
-      <c r="M75" t="inlineStr"/>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>54386711</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>127.97</t>
+        </is>
+      </c>
       <c r="N75" t="inlineStr"/>
     </row>
     <row r="76">
@@ -4482,8 +4534,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L76" t="inlineStr"/>
-      <c r="M76" t="inlineStr"/>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>54387666</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>121.49</t>
+        </is>
+      </c>
       <c r="N76" t="inlineStr"/>
     </row>
     <row r="77">
@@ -4528,8 +4588,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L77" t="inlineStr"/>
-      <c r="M77" t="inlineStr"/>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>54387725</t>
+        </is>
+      </c>
+      <c r="M77" t="inlineStr">
+        <is>
+          <t>120.48</t>
+        </is>
+      </c>
       <c r="N77" t="inlineStr"/>
     </row>
     <row r="78">
@@ -4574,8 +4642,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L78" t="inlineStr"/>
-      <c r="M78" t="inlineStr"/>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>54387783</t>
+        </is>
+      </c>
+      <c r="M78" t="inlineStr">
+        <is>
+          <t>121.13</t>
+        </is>
+      </c>
       <c r="N78" t="inlineStr"/>
     </row>
     <row r="79">
@@ -4620,8 +4696,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L79" t="inlineStr"/>
-      <c r="M79" t="inlineStr"/>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>54387838</t>
+        </is>
+      </c>
+      <c r="M79" t="inlineStr">
+        <is>
+          <t>113.59</t>
+        </is>
+      </c>
       <c r="N79" t="inlineStr"/>
     </row>
     <row r="80">
@@ -4666,8 +4750,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L80" t="inlineStr"/>
-      <c r="M80" t="inlineStr"/>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>54387898</t>
+        </is>
+      </c>
+      <c r="M80" t="inlineStr">
+        <is>
+          <t>121.43</t>
+        </is>
+      </c>
       <c r="N80" t="inlineStr"/>
     </row>
     <row r="81">
@@ -4712,8 +4804,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L81" t="inlineStr"/>
-      <c r="M81" t="inlineStr"/>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>54387947</t>
+        </is>
+      </c>
+      <c r="M81" t="inlineStr">
+        <is>
+          <t>114.89</t>
+        </is>
+      </c>
       <c r="N81" t="inlineStr"/>
     </row>
     <row r="82">
@@ -4758,8 +4858,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L82" t="inlineStr"/>
-      <c r="M82" t="inlineStr"/>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>54387993</t>
+        </is>
+      </c>
+      <c r="M82" t="inlineStr">
+        <is>
+          <t>113.63</t>
+        </is>
+      </c>
       <c r="N82" t="inlineStr"/>
     </row>
     <row r="83">
@@ -4804,8 +4912,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L83" t="inlineStr"/>
-      <c r="M83" t="inlineStr"/>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>54388066</t>
+        </is>
+      </c>
+      <c r="M83" t="inlineStr">
+        <is>
+          <t>114.29</t>
+        </is>
+      </c>
       <c r="N83" t="inlineStr"/>
     </row>
     <row r="84">
@@ -4850,8 +4966,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L84" t="inlineStr"/>
-      <c r="M84" t="inlineStr"/>
+      <c r="L84" t="inlineStr">
+        <is>
+          <t>54388111</t>
+        </is>
+      </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>117.93</t>
+        </is>
+      </c>
       <c r="N84" t="inlineStr"/>
     </row>
     <row r="85">
@@ -4896,8 +5020,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L85" t="inlineStr"/>
-      <c r="M85" t="inlineStr"/>
+      <c r="L85" t="inlineStr">
+        <is>
+          <t>54388153</t>
+        </is>
+      </c>
+      <c r="M85" t="inlineStr">
+        <is>
+          <t>114.52</t>
+        </is>
+      </c>
       <c r="N85" t="inlineStr"/>
     </row>
     <row r="86">
@@ -4942,8 +5074,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
-      <c r="M86" t="inlineStr"/>
+      <c r="L86" t="inlineStr">
+        <is>
+          <t>54388230</t>
+        </is>
+      </c>
+      <c r="M86" t="inlineStr">
+        <is>
+          <t>114.27</t>
+        </is>
+      </c>
       <c r="N86" t="inlineStr"/>
     </row>
     <row r="87">
@@ -4988,8 +5128,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
-      <c r="M87" t="inlineStr"/>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>54388276</t>
+        </is>
+      </c>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>114.55</t>
+        </is>
+      </c>
       <c r="N87" t="inlineStr"/>
     </row>
     <row r="88">
@@ -5034,8 +5182,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr"/>
-      <c r="M88" t="inlineStr"/>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>DOCUMENTO NO APLICA PARA ACTIVACIÓN POLIEDRO</t>
+        </is>
+      </c>
       <c r="N88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -5080,8 +5236,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L89" t="inlineStr"/>
-      <c r="M89" t="inlineStr"/>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>54388497</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>121.98</t>
+        </is>
+      </c>
       <c r="N89" t="inlineStr"/>
     </row>
     <row r="90">
@@ -5126,8 +5290,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr"/>
-      <c r="M90" t="inlineStr"/>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>54388583</t>
+        </is>
+      </c>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>132.03</t>
+        </is>
+      </c>
       <c r="N90" t="inlineStr"/>
     </row>
     <row r="91">
@@ -5172,8 +5344,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
-      <c r="M91" t="inlineStr"/>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>54388653</t>
+        </is>
+      </c>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>128.83</t>
+        </is>
+      </c>
       <c r="N91" t="inlineStr"/>
     </row>
     <row r="92">
@@ -5218,8 +5398,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L92" t="inlineStr"/>
-      <c r="M92" t="inlineStr"/>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>54388719</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>119.19</t>
+        </is>
+      </c>
       <c r="N92" t="inlineStr"/>
     </row>
     <row r="93">
@@ -5264,8 +5452,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
-      <c r="M93" t="inlineStr"/>
+      <c r="L93" t="inlineStr">
+        <is>
+          <t>54388784</t>
+        </is>
+      </c>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>119.6</t>
+        </is>
+      </c>
       <c r="N93" t="inlineStr"/>
     </row>
     <row r="94">
@@ -5310,8 +5506,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
-      <c r="M94" t="inlineStr"/>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>54388833</t>
+        </is>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>129.91</t>
+        </is>
+      </c>
       <c r="N94" t="inlineStr"/>
     </row>
     <row r="95">
@@ -5356,8 +5560,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>54388895</t>
+        </is>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>117.99</t>
+        </is>
+      </c>
       <c r="N95" t="inlineStr"/>
     </row>
     <row r="96">
@@ -5402,8 +5614,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>54388952</t>
+        </is>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>116.16</t>
+        </is>
+      </c>
       <c r="N96" t="inlineStr"/>
     </row>
     <row r="97">
@@ -5448,8 +5668,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>54389016</t>
+        </is>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>129.36</t>
+        </is>
+      </c>
       <c r="N97" t="inlineStr"/>
     </row>
     <row r="98">
@@ -5494,8 +5722,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>54389069</t>
+        </is>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>127.04</t>
+        </is>
+      </c>
       <c r="N98" t="inlineStr"/>
     </row>
     <row r="99">
@@ -5540,8 +5776,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>54389137</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>124.38</t>
+        </is>
+      </c>
       <c r="N99" t="inlineStr"/>
     </row>
     <row r="100">
@@ -5586,8 +5830,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>54391768</t>
+        </is>
+      </c>
+      <c r="M100" t="inlineStr">
+        <is>
+          <t>112.98</t>
+        </is>
+      </c>
       <c r="N100" t="inlineStr"/>
     </row>
     <row r="101">
@@ -5632,8 +5884,16 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>54391276</t>
+        </is>
+      </c>
+      <c r="M101" t="inlineStr">
+        <is>
+          <t>109.48</t>
+        </is>
+      </c>
       <c r="N101" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Se realizan pruebas de Portas y se despliega versión 3.6.14
</commit_message>
<xml_diff>
--- a/src/portas/portabilidad.xlsx
+++ b/src/portas/portabilidad.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,37 +506,37 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1001881631</v>
+        <v>16674113</v>
       </c>
       <c r="B2" s="2" t="n">
-        <v>43858</v>
+        <v>29532</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MILEIDIS</t>
+          <t>Oscar Emilio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> GUTIÉRREZ MENDOZA</t>
+          <t>Rivera Atehortua</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3006616218</v>
+        <v>3137047543</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702607221914</t>
+          <t xml:space="preserve"> 57101702606777550</t>
         </is>
       </c>
       <c r="G2" t="n">
-        <v>3217390710</v>
+        <v>3145406847</v>
       </c>
       <c r="H2" t="n">
         <v>1128390723</v>
       </c>
       <c r="I2" t="n">
-        <v>75063</v>
+        <v>79134</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -550,49 +550,49 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>54954372</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>117.44</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1091884029</v>
+        <v>14802083</v>
       </c>
       <c r="B3" s="2" t="n">
-        <v>44553</v>
+        <v>38000</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>JOSE LUIS</t>
+          <t>ANDRES</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MORA BARRERO</t>
+          <t>ANDRES MONCAYO</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3015511578</v>
+        <v>3046360017</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411371517</t>
+          <t xml:space="preserve"> 57101702411459870</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>3235789939</v>
+        <v>3126383897</v>
       </c>
       <c r="H3" t="n">
         <v>1128390723</v>
       </c>
       <c r="I3" t="n">
-        <v>53127</v>
+        <v>24144</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -606,49 +606,49 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>54954399</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>123.24</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1091884029</v>
+        <v>14802083</v>
       </c>
       <c r="B4" s="2" t="n">
-        <v>44553</v>
+        <v>38000</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>JOSE LUIS</t>
+          <t>ANDRES</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MORA BARRERO</t>
+          <t>ANDRES MONCAYO</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3015510666</v>
+        <v>3046049958</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411371510</t>
+          <t xml:space="preserve"> 57101702411459869</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>3235789956</v>
+        <v>3126386442</v>
       </c>
       <c r="H4" t="n">
         <v>1128390723</v>
       </c>
       <c r="I4" t="n">
-        <v>68667</v>
+        <v>46088</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -662,49 +662,49 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>54954422</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>116.84</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1091884029</v>
+        <v>15209170</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>44553</v>
+        <v>37951</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>JOSE LUIS</t>
+          <t>ALEXIS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MORA BARRERO</t>
+          <t>MIRANDA EXTRADA</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3015511557</v>
+        <v>3046363852</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411400506</t>
+          <t xml:space="preserve"> 57101702411459867</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>3235845946</v>
+        <v>3126387718</v>
       </c>
       <c r="H5" t="n">
         <v>1128390723</v>
       </c>
       <c r="I5" t="n">
-        <v>97802</v>
+        <v>55759</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -723,44 +723,44 @@
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>El numero 3046363852 no tiene solicitud de NIP Vigente</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>71787091</v>
+        <v>15209170</v>
       </c>
       <c r="B6" s="2" t="n">
-        <v>34846</v>
+        <v>37951</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JULIAN DAVID</t>
+          <t>ALEXI</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MC LEAN RAMOS</t>
+          <t>MIRANDA ESTRADA</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3015510924</v>
+        <v>3046354471</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411371511</t>
+          <t xml:space="preserve"> 57101702411459865</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>3235789951</v>
+        <v>3126416751</v>
       </c>
       <c r="H6" t="n">
         <v>1128390723</v>
       </c>
       <c r="I6" t="n">
-        <v>72353</v>
+        <v>99215</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -774,49 +774,49 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>54954474</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>122.57</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>71787091</v>
+        <v>15209332</v>
       </c>
       <c r="B7" s="2" t="n">
-        <v>34846</v>
+        <v>37991</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JULIAN DAVID</t>
+          <t>CRISTIAN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MC LEAN RAMOS</t>
+          <t>PABON ALVAREZ</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3015511586</v>
+        <v>3126427443</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411459810</t>
+          <t xml:space="preserve"> 57101712411459864</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>3126160262</v>
+        <v>3126427443</v>
       </c>
       <c r="H7" t="n">
         <v>1128390723</v>
       </c>
       <c r="I7" t="n">
-        <v>97908</v>
+        <v>7647</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -835,44 +835,44 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>El ICCID "712411459864" no existe en SAP, si el equipo es del cliente marque la opción de Trajo ICCID.</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>71787091</v>
+        <v>14801180</v>
       </c>
       <c r="B8" s="2" t="n">
-        <v>34846</v>
+        <v>37768</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>JULIAN DAVID</t>
+          <t>JESUS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> MC LEAN RAMOS</t>
+          <t>BLANCO GARCIA</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3015510709</v>
+        <v>3046356303</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411459809</t>
+          <t xml:space="preserve"> 57101702411375956</t>
         </is>
       </c>
       <c r="G8" t="n">
-        <v>3126160289</v>
+        <v>3235856464</v>
       </c>
       <c r="H8" t="n">
         <v>1128390723</v>
       </c>
       <c r="I8" t="n">
-        <v>15991</v>
+        <v>93280</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -886,49 +886,49 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>error</t>
+          <t>54954512</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
+          <t>117.82</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1037581400</v>
+        <v>14801180</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>38517</v>
+        <v>37768</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MARIA JOHANA</t>
+          <t>JESUS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> RAMIREZ FRANCO</t>
+          <t>BLANCO GARCIA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3015510792</v>
+        <v>3046048778</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702411459808</t>
+          <t xml:space="preserve"> 57101702607176622</t>
         </is>
       </c>
       <c r="G9" t="n">
-        <v>3126161381</v>
+        <v>3136480485</v>
       </c>
       <c r="H9" t="n">
         <v>1128390723</v>
       </c>
       <c r="I9" t="n">
-        <v>19931</v>
+        <v>69839</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -942,15 +942,295 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
+          <t>54954528</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>113.71</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>14802064</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>36900</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>DIDIER</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>VILLEGAS MONTES</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>3001763840</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702503210838</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>3233263551</v>
+      </c>
+      <c r="H10" t="n">
+        <v>1128390723</v>
+      </c>
+      <c r="I10" t="n">
+        <v>91756</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>master.33@gmail.com</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>prepago</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
           <t>error</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
-        <is>
-          <t>El ICCID se encuentra en un proceso de activación en curso</t>
-        </is>
-      </c>
-      <c r="N9" t="inlineStr"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>La Dupla ICCID - MSISDN NO corresponde, no se puede continuar con la Activacion.</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>14802064</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>45666</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>DIDIER</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>VILLEGAS MONTES</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>3046353992</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702503210837</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>3233266458</v>
+      </c>
+      <c r="H11" t="n">
+        <v>1128390723</v>
+      </c>
+      <c r="I11" t="n">
+        <v>49699</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>master.33@gmail.com</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>prepago</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>error</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>La Dupla ICCID - MSISDN NO corresponde, no se puede continuar con la Activacion.</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>14802064</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>37995</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>DIDIER</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>VILLEGAS MONTES</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>3001763587</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702503249730</t>
+        </is>
+      </c>
+      <c r="G12" t="n">
+        <v>3234255358</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1128390723</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2661</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>master.33@gmail.com</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>prepago</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>54954595</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>117.64</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>14802064</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>37995</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>DIDIER</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>VILLEGAS MONTES</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>3046354130</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702503249729</t>
+        </is>
+      </c>
+      <c r="G13" t="n">
+        <v>3234255396</v>
+      </c>
+      <c r="H13" t="n">
+        <v>1128390723</v>
+      </c>
+      <c r="I13" t="n">
+        <v>16778</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>master.33@gmail.com</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>prepago</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>54954619</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>121.5</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>14802083</v>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>38000</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>ANDRES</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>ANDRES MONCAYO</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3046353586</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 57101702503249728</t>
+        </is>
+      </c>
+      <c r="G14" t="n">
+        <v>3234256628</v>
+      </c>
+      <c r="H14" t="n">
+        <v>1128390723</v>
+      </c>
+      <c r="I14" t="n">
+        <v>77357</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>master.33@gmail.com</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>prepago</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>54954647</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>109.95</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Seleccionar acceso correcto despues de re-login
</commit_message>
<xml_diff>
--- a/src/portas/portabilidad.xlsx
+++ b/src/portas/portabilidad.xlsx
@@ -506,29 +506,27 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>1114091053</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1128051223</v>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>38371</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>JOHN</t>
+          <t>GIOVANY</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>GALINDO</t>
+          <t>LOPEZ SOLANO</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>3244371133</v>
+        <v>3006196447</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650122</t>
+          <t xml:space="preserve"> 57101702502408750</t>
         </is>
       </c>
       <c r="G2" t="inlineStr"/>
@@ -536,7 +534,7 @@
         <v>1128390723</v>
       </c>
       <c r="I2" t="n">
-        <v>56723</v>
+        <v>99680</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -550,41 +548,39 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>56735436</t>
+          <t>56796230</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>186.01</t>
+          <t>162.66</t>
         </is>
       </c>
       <c r="N2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>1082909870</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1001818090</v>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>39700</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>BERTA</t>
+          <t>BRAYAN</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>GUERRERO</t>
+          <t>MUNIVE RANGEL</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>3244121129</v>
+        <v>3244142203</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650480</t>
+          <t xml:space="preserve"> 57101702502408754</t>
         </is>
       </c>
       <c r="G3" t="inlineStr"/>
@@ -592,7 +588,7 @@
         <v>1128390723</v>
       </c>
       <c r="I3" t="n">
-        <v>26548</v>
+        <v>28713</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -606,41 +602,39 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>56735544</t>
+          <t>56796314</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>188.82</t>
+          <t>160.84</t>
         </is>
       </c>
       <c r="N3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>1128401707</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1130588130</v>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>38282</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>EDISON</t>
+          <t>FANNY</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>OCAMPO</t>
+          <t>TORRES TREJOS</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>3007120061</v>
+        <v>3244136345</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650481</t>
+          <t xml:space="preserve"> 57101702502408756</t>
         </is>
       </c>
       <c r="G4" t="inlineStr"/>
@@ -648,7 +642,7 @@
         <v>1128390723</v>
       </c>
       <c r="I4" t="n">
-        <v>17911</v>
+        <v>50864</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -662,39 +656,39 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>56735776</t>
+          <t>56796413</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>189.54</t>
+          <t>169.21</t>
         </is>
       </c>
       <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1094269187</v>
+        <v>1022972942</v>
       </c>
       <c r="B5" s="2" t="n">
-        <v>40410</v>
+        <v>40158</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KELLY</t>
+          <t>YHONNY</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>PAEZ</t>
+          <t>BARON RIVERA</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>3246739533</v>
+        <v>3007116763</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650482</t>
+          <t xml:space="preserve"> 57101702502408758</t>
         </is>
       </c>
       <c r="G5" t="inlineStr"/>
@@ -702,7 +696,7 @@
         <v>1128390723</v>
       </c>
       <c r="I5" t="n">
-        <v>98522</v>
+        <v>69379</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -716,41 +710,39 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>56735880</t>
+          <t>56796507</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>191.79</t>
+          <t>167.73</t>
         </is>
       </c>
       <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1018455899</v>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1087194318</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>40498</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>JAIR</t>
+          <t>DELIA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>MOYA</t>
+          <t>MONSALVE CABEZAS</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>3001921350</v>
+        <v>3244120440</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650483</t>
+          <t xml:space="preserve"> 57101702502408898</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -758,7 +750,7 @@
         <v>1128390723</v>
       </c>
       <c r="I6" t="n">
-        <v>48548</v>
+        <v>32527</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -772,41 +764,39 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>56735957</t>
+          <t>56796605</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>159.03</t>
+          <t>178.42</t>
         </is>
       </c>
       <c r="N6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1143841277</v>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1106738115</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>38140</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>JUAN</t>
+          <t>MARIA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>BETANCOURT</t>
+          <t>ARIAS VERGARA</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>3244373131</v>
+        <v>3244133259</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650523</t>
+          <t xml:space="preserve"> 57101702502408900</t>
         </is>
       </c>
       <c r="G7" t="inlineStr"/>
@@ -814,7 +804,7 @@
         <v>1128390723</v>
       </c>
       <c r="I7" t="n">
-        <v>281</v>
+        <v>33347</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -828,41 +818,39 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>56736051</t>
+          <t>56796694</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>187.61</t>
+          <t>165.15</t>
         </is>
       </c>
       <c r="N7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1100960031</v>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1106771241</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>38526</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>CARLOS</t>
+          <t>YURY</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>IBARRA</t>
+          <t>ACUÑA MORALES</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>3001889467</v>
+        <v>3244136607</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650524</t>
+          <t xml:space="preserve"> 57101702502408901</t>
         </is>
       </c>
       <c r="G8" t="inlineStr"/>
@@ -870,7 +858,7 @@
         <v>1128390723</v>
       </c>
       <c r="I8" t="n">
-        <v>43471</v>
+        <v>53844</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -884,39 +872,39 @@
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>56736111</t>
+          <t>56796769</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>164.01</t>
+          <t>174.82</t>
         </is>
       </c>
       <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1015436600</v>
+        <v>1110504013</v>
       </c>
       <c r="B9" s="2" t="n">
-        <v>40585</v>
+        <v>39772</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LUIS</t>
+          <t>PAULA</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>RODRIGUEZ</t>
+          <t>LOMBANA SIERRA</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3004842229</v>
+        <v>3244122199</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650525</t>
+          <t xml:space="preserve"> 57101702502408927</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
@@ -924,7 +912,7 @@
         <v>1128390723</v>
       </c>
       <c r="I9" t="n">
-        <v>97439</v>
+        <v>91570</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -938,41 +926,39 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>56736189</t>
+          <t>56796888</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>163.58</t>
+          <t>162.68</t>
         </is>
       </c>
       <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1098713747</v>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Sin</t>
-        </is>
+        <v>1121862409</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>39534</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>JHON</t>
+          <t>RUTH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>FUENTES</t>
+          <t>OLARTE VERA</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>3016025451</v>
+        <v>3007126561</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650526</t>
+          <t xml:space="preserve"> 57101702502408934</t>
         </is>
       </c>
       <c r="G10" t="inlineStr"/>
@@ -980,7 +966,7 @@
         <v>1128390723</v>
       </c>
       <c r="I10" t="n">
-        <v>5404</v>
+        <v>53115</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -992,41 +978,37 @@
           <t>prepago</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
-        <is>
-          <t>56736256</t>
-        </is>
-      </c>
+      <c r="L10" t="inlineStr"/>
       <c r="M10" t="inlineStr">
         <is>
-          <t>160.49</t>
+          <t>error</t>
         </is>
       </c>
       <c r="N10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>1072961831</v>
+        <v>1022366393</v>
       </c>
       <c r="B11" s="2" t="n">
-        <v>40337</v>
+        <v>39836</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>PAOLA</t>
+          <t>DIANA</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>JUTINICO</t>
+          <t>HERRERA CARRION</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>3016048217</v>
+        <v>3004843216</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 57101702507650527</t>
+          <t xml:space="preserve"> 57101702502408938</t>
         </is>
       </c>
       <c r="G11" t="inlineStr"/>
@@ -1034,7 +1016,7 @@
         <v>1128390723</v>
       </c>
       <c r="I11" t="n">
-        <v>34301</v>
+        <v>70924</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1047,11 +1029,7 @@
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr">
-        <is>
-          <t>error</t>
-        </is>
-      </c>
+      <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
     </row>
     <row r="12">

</xml_diff>